<commit_message>
Se agrego el llamado proyecto RH_Templates desde pdnink
</commit_message>
<xml_diff>
--- a/HR_Templates/wwwroot/signatures/ExcelGenerado.xlsx
+++ b/HR_Templates/wwwroot/signatures/ExcelGenerado.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\github\Portafoliodenegocios\HR_Templates\App_Data\b6cc7d08-501f-4dee-99c0-414c5df38672\Templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\github\Portafoliodenegocios\HR_Templates\App_Data\ebf91bd5-a22b-47ed-ba06-26bfdf64c58f\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -60,7 +60,7 @@
     <t>NOMBRE DEL EMPLEADO</t>
   </si>
   <si>
-    <t>david remiso</t>
+    <t>GFDGDFG</t>
   </si>
   <si>
     <t>N° DE NÓMINA</t>
@@ -78,7 +78,7 @@
     <t>PUESTO</t>
   </si>
   <si>
-    <t>Develepoer</t>
+    <t>DFG</t>
   </si>
   <si>
     <t>ÁREA A LA QUE PERTENECE</t>

</xml_diff>